<commit_message>
Improve Finnish history distractors
</commit_message>
<xml_diff>
--- a/kahoot/orientation/finnish-history/main-periods-of-finnish-history-1-finland-as-a-part-of-sweden-and-russia__0001.xlsx
+++ b/kahoot/orientation/finnish-history/main-periods-of-finnish-history-1-finland-as-a-part-of-sweden-and-russia__0001.xlsx
@@ -1897,12 +1897,12 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Islam</t>
+          <t>Luthersk kristendom</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>Buddhism</t>
+          <t>Reformert kristendom</t>
         </is>
       </c>
       <c r="G10" s="14" t="n">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Kommunfullmäktige</t>
+          <t>Kungliga rådet</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
@@ -1954,12 +1954,12 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Landstinget</t>
+          <t>Tvåkammarriksdagen</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Senaten</t>
+          <t>Riksrådet</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Alla vuxna med rösträtt</t>
+          <t>Jordägare och borgare med privilegier</t>
         </is>
       </c>
       <c r="G13" s="14" t="n">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>De bytte stånd varje år</t>
+          <t>De kunde ibland byta stånd genom giftermål</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>De tillhörde alltid adeln</t>
+          <t>De kunde byta stånd genom utbildning</t>
         </is>
       </c>
       <c r="G14" s="14" t="n">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>De blev alltid kvar hemma</t>
+          <t>De stred i lokala finska regementen</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>De blev automatiskt officerare</t>
+          <t>De tjänstgjorde ofta som sjömän och artillerister</t>
         </is>
       </c>
       <c r="G15" s="14" t="n">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>Den privatiserades helt</t>
+          <t>Den såldes till privata ägare</t>
         </is>
       </c>
       <c r="G20" s="14" t="n">
@@ -2514,12 +2514,12 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>Bara religiöst</t>
+          <t>Både religiöst och ekonomiskt</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>Bara ekonomiskt</t>
+          <t>Både religiöst och kulturellt</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Bara militärt</t>
+          <t>Både ekonomiskt och militärt</t>
         </is>
       </c>
       <c r="G21" s="14" t="n">
@@ -2747,17 +2747,17 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>Förbud mot resor</t>
+          <t>Stärkt statskyrka</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Tvångsarbete</t>
+          <t>Religiös enhet genom tvång</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>Förbud mot utbildning</t>
+          <t>Kyrkans makt ökade</t>
         </is>
       </c>
       <c r="G25" s="14" t="n">
@@ -2804,17 +2804,17 @@
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Total monarki</t>
+          <t>Rösträtt med egendomskrav</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Förbud mot val</t>
+          <t>Rösträtt för män</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Ståndssamhälle för alla</t>
+          <t>Rösträtt för höginkomsttagare</t>
         </is>
       </c>
       <c r="G26" s="14" t="n">

</xml_diff>